<commit_message>
Cuadro closer senior: 8% + 10% acelerador; cuadro objetivo de ingreso -> contratos
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/CUADRO_INGRESO_CLOSER_SENIOR.xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/CUADRO_INGRESO_CLOSER_SENIOR.xlsx
@@ -98,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -115,6 +115,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -481,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P34"/>
+  <dimension ref="A1:P42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -512,7 +513,7 @@
     <row r="2" ht="75" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>REGLAS. Meta: contratos firmados con la inicial pagada (mes 1: 6 · mes 2 y 3: 8 · meses 4-6: 10 · desde el mes 7: 12). Básico $2.000.000 (sube a $2.300.000 en el mes 4 y a $2.600.000 en el mes 7, por resultados). Bono de arranque meses 1 y 2: $1.500.000, se SUMA a la comisión, con condición: 5 citas atendidas por semana y al menos la mitad de la meta (3 contratos el mes 1, 4 el mes 2). Comisión: 7% del RECAUDO desde la primera venta (3,5% si es cliente antiguo) = $209,300 por cada matrícula de $2,990,000 pagada completa; si es a cuotas, la comisión entra mes a mes mientras el cliente paga. La celda sombreada es la meta.</t>
+          <t>REGLAS. Meta: contratos firmados con la inicial pagada (mes 1: 6 · mes 2 y 3: 8 · meses 4-6: 10 · desde el mes 7: 12). Básico $2.000.000 (sube a $2.300.000 en el mes 4 y a $2.600.000 en el mes 7, por resultados). Bono de arranque meses 1 y 2: $1.500.000, se SUMA a la comisión, con condición: 5 citas atendidas por semana y al menos la mitad de la meta (3 contratos el mes 1, 4 el mes 2). Comisión: 8% del RECAUDO desde la primera venta (= $239,200 por matrícula de $2,990,000 pagada completa) y 10% sobre lo que cierre por encima de la meta del mes (= $299,000); 4% si es cliente antiguo. Si es a cuotas, la comisión entra mes a mes mientras el cliente paga. La celda sombreada es la meta.</t>
         </is>
       </c>
     </row>
@@ -621,40 +622,40 @@
         <v>2000000</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>2209300</v>
+        <v>2239200</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>2418600</v>
+        <v>2478400</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>4127900</v>
+        <v>4217600</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>4337200</v>
+        <v>4456800</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>4546500</v>
+        <v>4696000</v>
       </c>
       <c r="J6" s="8" t="n">
-        <v>4755800</v>
+        <v>4935200</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>4965100</v>
+        <v>5234200</v>
       </c>
       <c r="L6" s="6" t="n">
-        <v>5174400</v>
+        <v>5533200</v>
       </c>
       <c r="M6" s="6" t="n">
-        <v>5383700</v>
+        <v>5832200</v>
       </c>
       <c r="N6" s="6" t="n">
-        <v>5593000</v>
+        <v>6131200</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>6011600</v>
+        <v>6729200</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>6639500</v>
+        <v>7626200</v>
       </c>
     </row>
     <row r="7">
@@ -673,40 +674,40 @@
         <v>2000000</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>2209300</v>
+        <v>2239200</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>2418600</v>
+        <v>2478400</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>2627900</v>
+        <v>2717600</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>4337200</v>
+        <v>4456800</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>4546500</v>
+        <v>4696000</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>4755800</v>
+        <v>4935200</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>4965100</v>
+        <v>5174400</v>
       </c>
       <c r="L7" s="8" t="n">
-        <v>5174400</v>
+        <v>5413600</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>5383700</v>
+        <v>5712600</v>
       </c>
       <c r="N7" s="6" t="n">
-        <v>5593000</v>
+        <v>6011600</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>6011600</v>
+        <v>6609600</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>6639500</v>
+        <v>7506600</v>
       </c>
     </row>
     <row r="8">
@@ -725,40 +726,40 @@
         <v>2000000</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>2209300</v>
+        <v>2239200</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>2418600</v>
+        <v>2478400</v>
       </c>
       <c r="G8" s="7" t="n">
-        <v>2627900</v>
+        <v>2717600</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>2837200</v>
+        <v>2956800</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>3046500</v>
+        <v>3196000</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>3255800</v>
+        <v>3435200</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>3465100</v>
+        <v>3674400</v>
       </c>
       <c r="L8" s="8" t="n">
-        <v>3674400</v>
+        <v>3913600</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>3883700</v>
+        <v>4212600</v>
       </c>
       <c r="N8" s="6" t="n">
-        <v>4093000</v>
+        <v>4511600</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>4511600</v>
+        <v>5109600</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>5139500</v>
+        <v>6006600</v>
       </c>
     </row>
     <row r="9">
@@ -777,40 +778,40 @@
         <v>2300000</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>2509300</v>
+        <v>2539200</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>2718600</v>
+        <v>2778400</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>2927900</v>
+        <v>3017600</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>3137200</v>
+        <v>3256800</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>3346500</v>
+        <v>3496000</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3555800</v>
+        <v>3735200</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>3765100</v>
+        <v>3974400</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>3974400</v>
+        <v>4213600</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>4183700</v>
+        <v>4452800</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>4393000</v>
+        <v>4692000</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>4811600</v>
+        <v>5290000</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>5439500</v>
+        <v>6187000</v>
       </c>
     </row>
     <row r="10">
@@ -829,46 +830,46 @@
         <v>2600000</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>2809300</v>
+        <v>2839200</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>3018600</v>
+        <v>3078400</v>
       </c>
       <c r="G10" s="7" t="n">
-        <v>3227900</v>
+        <v>3317600</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>3437200</v>
+        <v>3556800</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>3646500</v>
+        <v>3796000</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>3855800</v>
+        <v>4035200</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>4065100</v>
+        <v>4274400</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>4274400</v>
+        <v>4513600</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>4483700</v>
+        <v>4752800</v>
       </c>
       <c r="N10" s="6" t="n">
-        <v>4693000</v>
+        <v>4992000</v>
       </c>
       <c r="O10" s="8" t="n">
-        <v>5111600</v>
+        <v>5470400</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>5739500</v>
+        <v>6367400</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Gris: por debajo de la mitad de la meta (en meses 1-2 no hay bono). Ejemplo mes 1 con 5 contratos: $2.000.000 + $1.500.000 + 5 x $209.300 = $4.546.500. Mes 1 con 2 contratos: $2.000.000 + 2 x $209.300 = $2.418.600 (sin bono).</t>
+          <t>Gris: por debajo de la mitad de la meta (en meses 1-2 no hay bono). Ejemplo mes 1 con 5 contratos: $2.000.000 + $1.500.000 + 5 x $239.200 = $4.696.000. Mes 1 con 2 contratos: $2.000.000 + 2 x $239.200 = $2.478.400 (sin bono). Por encima de la meta cada contrato vale $299.000.</t>
         </is>
       </c>
     </row>
@@ -907,7 +908,7 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>Comisión del mes (7%)</t>
+          <t>Comisión del mes (8%)</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
@@ -945,7 +946,7 @@
         <v>7200000</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>504000.0000000001</v>
+        <v>576000</v>
       </c>
       <c r="G15" s="6" t="n">
         <v>1500000</v>
@@ -954,7 +955,7 @@
         <v>2000000</v>
       </c>
       <c r="I15" s="8" t="n">
-        <v>4004000</v>
+        <v>4076000</v>
       </c>
     </row>
     <row r="16">
@@ -976,7 +977,7 @@
         <v>12300000</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>861000.0000000001</v>
+        <v>984000</v>
       </c>
       <c r="G16" s="6" t="n">
         <v>1500000</v>
@@ -985,7 +986,7 @@
         <v>2000000</v>
       </c>
       <c r="I16" s="8" t="n">
-        <v>4361000</v>
+        <v>4484000</v>
       </c>
     </row>
     <row r="17">
@@ -1007,7 +1008,7 @@
         <v>15900000</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>1113000</v>
+        <v>1272000</v>
       </c>
       <c r="G17" s="6" t="n">
         <v>0</v>
@@ -1016,7 +1017,7 @@
         <v>2000000</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>3113000</v>
+        <v>3272000</v>
       </c>
     </row>
     <row r="18">
@@ -1038,7 +1039,7 @@
         <v>21900000</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>1533000</v>
+        <v>1752000</v>
       </c>
       <c r="G18" s="6" t="n">
         <v>0</v>
@@ -1047,7 +1048,7 @@
         <v>2300000</v>
       </c>
       <c r="I18" s="8" t="n">
-        <v>3833000</v>
+        <v>4052000</v>
       </c>
     </row>
     <row r="19">
@@ -1069,7 +1070,7 @@
         <v>26400000</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>1848000</v>
+        <v>2112000</v>
       </c>
       <c r="G19" s="6" t="n">
         <v>0</v>
@@ -1078,7 +1079,7 @@
         <v>2300000</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>4148000</v>
+        <v>4412000</v>
       </c>
     </row>
     <row r="20">
@@ -1100,7 +1101,7 @@
         <v>28200000</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>1974000</v>
+        <v>2256000</v>
       </c>
       <c r="G20" s="6" t="n">
         <v>0</v>
@@ -1109,7 +1110,7 @@
         <v>2300000</v>
       </c>
       <c r="I20" s="8" t="n">
-        <v>4274000</v>
+        <v>4556000</v>
       </c>
     </row>
     <row r="21">
@@ -1131,7 +1132,7 @@
         <v>31500000</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>2205000</v>
+        <v>2520000</v>
       </c>
       <c r="G21" s="6" t="n">
         <v>0</v>
@@ -1140,7 +1141,7 @@
         <v>2600000</v>
       </c>
       <c r="I21" s="8" t="n">
-        <v>4805000</v>
+        <v>5120000</v>
       </c>
     </row>
     <row r="22">
@@ -1162,7 +1163,7 @@
         <v>33300000</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>2331000</v>
+        <v>2664000</v>
       </c>
       <c r="G22" s="6" t="n">
         <v>0</v>
@@ -1171,7 +1172,7 @@
         <v>2600000</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>4931000</v>
+        <v>5264000</v>
       </c>
     </row>
     <row r="23">
@@ -1193,7 +1194,7 @@
         <v>34200000</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>2394000</v>
+        <v>2736000</v>
       </c>
       <c r="G23" s="6" t="n">
         <v>0</v>
@@ -1202,7 +1203,7 @@
         <v>2600000</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>4994000</v>
+        <v>5336000</v>
       </c>
     </row>
     <row r="24">
@@ -1224,7 +1225,7 @@
         <v>35100000</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>2457000</v>
+        <v>2808000</v>
       </c>
       <c r="G24" s="6" t="n">
         <v>0</v>
@@ -1233,7 +1234,7 @@
         <v>2600000</v>
       </c>
       <c r="I24" s="8" t="n">
-        <v>5057000</v>
+        <v>5408000</v>
       </c>
     </row>
     <row r="25">
@@ -1255,7 +1256,7 @@
         <v>36000000</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>2520000</v>
+        <v>2880000</v>
       </c>
       <c r="G25" s="6" t="n">
         <v>0</v>
@@ -1264,7 +1265,7 @@
         <v>2600000</v>
       </c>
       <c r="I25" s="8" t="n">
-        <v>5120000</v>
+        <v>5480000</v>
       </c>
     </row>
     <row r="26">
@@ -1286,7 +1287,7 @@
         <v>36000000</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>2520000</v>
+        <v>2880000</v>
       </c>
       <c r="G26" s="6" t="n">
         <v>0</v>
@@ -1295,7 +1296,7 @@
         <v>2600000</v>
       </c>
       <c r="I26" s="8" t="n">
-        <v>5120000</v>
+        <v>5480000</v>
       </c>
     </row>
     <row r="27" ht="45" customHeight="1">
@@ -1306,42 +1307,141 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>CUADRO 3 — PARA GANAR X, CUÁNTOS CONTRATOS NECESITA (de contado; desde el mes 3, sin bono)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>Quiere ganar</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Mes 3 (básico $2.0M, meta 8)</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Meses 4-6 (básico $2.3M, meta 10)</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Desde el mes 7 (básico $2.6M, meta 12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
         <is>
           <t>LO QUE ARRIESGA LA ACADEMIA Y LAS CONDICIONES</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t>• Si no vende nada: solo el básico ($2.000.000 al mes); el bono de arranque exige la mitad de la meta, así que no se paga con 0 ventas.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>• Peor caso con bono: meses 1 y 2 a media meta (3 y 4 contratos): $3.500.000 + comisión de 3 y 4 contratos. Todo lo demás sale de ventas ya cobradas.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>• Condiciones: prueba práctica de cierre antes de firmar; período de prueba de 2 meses (coincide con el bono); metas y mediciones del REGLAMENTO_MEDICION_COMERCIAL (este rol tiene su propia curva: 6/8/8/10/12 y comisión desde la primera venta); ascensos de básico solo por resultados.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>• Condiciones: prueba práctica de cierre antes de firmar; período de prueba de 2 meses (coincide con el bono); metas y mediciones del REGLAMENTO_MEDICION_COMERCIAL (este rol tiene su propia curva: 6/8/8/10/12, comisión 8% desde la primera venta y 10% por encima de la meta); ascensos de básico solo por resultados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>• Empresas que ella abra (fuera del piloto docente): 3% del recaudo corporativo del primer año.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>• Frontera con la asesora actual (comisión pura): citas del asistente y franjas que la asesora no cubre van a la closer; canales propios de cada una se respetan; la comisión es de quien atiende y cierra.</t>
         </is>
@@ -1350,12 +1450,12 @@
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A11:P11"/>
-    <mergeCell ref="A32:P32"/>
+    <mergeCell ref="A42:P42"/>
+    <mergeCell ref="A40:P40"/>
     <mergeCell ref="A27:P27"/>
-    <mergeCell ref="A31:P31"/>
-    <mergeCell ref="A34:P34"/>
-    <mergeCell ref="A30:P30"/>
-    <mergeCell ref="A33:P33"/>
+    <mergeCell ref="A39:P39"/>
+    <mergeCell ref="A38:P38"/>
+    <mergeCell ref="A41:P41"/>
     <mergeCell ref="A2:P2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Closer senior: hoja de reglas de conteo por tipo de venta y economia para la academia
</commit_message>
<xml_diff>
--- a/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/CUADRO_INGRESO_CLOSER_SENIOR.xlsx
+++ b/recursos/comercial/INDUCCION_COMERCIAL/contratacion comercial/CUADRO_INGRESO_CLOSER_SENIOR.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INGRESO" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TABLERO SEMANAL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REGLAS DE CONTEO" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TABLERO SEMANAL" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,10 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +50,9 @@
     <font>
       <b val="1"/>
       <color rgb="00E54C09"/>
+    </font>
+    <font>
+      <i val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -99,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -118,6 +123,12 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1457,6 +1468,335 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CÓMO CUENTA CADA TIPO DE VENTA (para la meta y para la comisión)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Tipo de venta</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>Cuenta para la meta</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>Comisión</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Programa completo de contado ($4.78M-$5.9M)</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>1 contrato</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>12% / 15% del recaudo, de una vez ($574k-$709k)</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Mejor venta posible</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Arranque de contado ($2.99M)</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1 contrato</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>$358.800 de una vez (12%)</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Cualquier programa a cuotas</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>1 contrato cuando la INICIAL está pagada (mínimo $1.000.000 o 30%)</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>12% de la inicial ese mes + 12% de cada cuota cuando entra</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>La cartera: comisión mes a mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Separación de $300.000 sola</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>0 (lead en proceso)</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>12% de los $300.000; el resto cuando pague la inicial</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>No llena la meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Nivel suelto / sabatino ($1.6M-$2.3M)</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>½ contrato</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>12% del recaudo</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Cliente antiguo (continuidad, supletorio)</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>½ contrato</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>6% del recaudo</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Plan empresa que ella abra (fuera del piloto docente)</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>1 contrato por cupo</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>3% del recaudo corporativo del primer año</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Gerencia firma</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Regla: la meta solo se cumple con programas con inicial pagada; separaciones y niveles sueltos no la llenan. La comisión siempre es sobre plata que entró.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>LO QUE RECIBE LA ACADEMIA (si fueran de contado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Contratos al mes</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>Recaudo</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>Comisión (12%/15%)</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Neto academia</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>% para ella</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>23920000</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>2870400</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>21049600</v>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>29900000</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>3588000</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>26312000</v>
+      </c>
+      <c r="E17" s="15" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>35880000</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>4305600</v>
+      </c>
+      <c r="D18" s="7" t="n">
+        <v>31574400</v>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>44850000</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>5651100</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>39198900</v>
+      </c>
+      <c r="E19" s="15" t="n">
+        <v>0.126</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>53820000</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>6996600</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>46823400</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>0.13</v>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>12 contratos al mes = la academia sana (~100 estudiantes pagando, ~$35M de caja). A cuotas, el recaudo del mes arranca en ~$14M de iniciales y llega a ~$36M hacia el quinto mes con la cartera; la comisión va igual de atrás.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A22:E22"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1553,7 +1893,7 @@
       <c r="F5" s="7" t="n"/>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
-      <c r="I5" s="12">
+      <c r="I5" s="16">
         <f>IF(H5="","",G5/H5)</f>
         <v/>
       </c>
@@ -1569,7 +1909,7 @@
       <c r="F6" s="7" t="n"/>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="n"/>
-      <c r="I6" s="12">
+      <c r="I6" s="16">
         <f>IF(H6="","",G6/H6)</f>
         <v/>
       </c>
@@ -1585,7 +1925,7 @@
       <c r="F7" s="7" t="n"/>
       <c r="G7" s="5" t="n"/>
       <c r="H7" s="5" t="n"/>
-      <c r="I7" s="12">
+      <c r="I7" s="16">
         <f>IF(H7="","",G7/H7)</f>
         <v/>
       </c>
@@ -1601,7 +1941,7 @@
       <c r="F8" s="7" t="n"/>
       <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="n"/>
-      <c r="I8" s="12">
+      <c r="I8" s="16">
         <f>IF(H8="","",G8/H8)</f>
         <v/>
       </c>
@@ -1617,7 +1957,7 @@
       <c r="F9" s="7" t="n"/>
       <c r="G9" s="5" t="n"/>
       <c r="H9" s="5" t="n"/>
-      <c r="I9" s="12">
+      <c r="I9" s="16">
         <f>IF(H9="","",G9/H9)</f>
         <v/>
       </c>
@@ -1633,7 +1973,7 @@
       <c r="F10" s="7" t="n"/>
       <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="n"/>
-      <c r="I10" s="12">
+      <c r="I10" s="16">
         <f>IF(H10="","",G10/H10)</f>
         <v/>
       </c>
@@ -1649,7 +1989,7 @@
       <c r="F11" s="7" t="n"/>
       <c r="G11" s="5" t="n"/>
       <c r="H11" s="5" t="n"/>
-      <c r="I11" s="12">
+      <c r="I11" s="16">
         <f>IF(H11="","",G11/H11)</f>
         <v/>
       </c>
@@ -1665,7 +2005,7 @@
       <c r="F12" s="7" t="n"/>
       <c r="G12" s="5" t="n"/>
       <c r="H12" s="5" t="n"/>
-      <c r="I12" s="12">
+      <c r="I12" s="16">
         <f>IF(H12="","",G12/H12)</f>
         <v/>
       </c>
@@ -1681,7 +2021,7 @@
       <c r="F13" s="7" t="n"/>
       <c r="G13" s="5" t="n"/>
       <c r="H13" s="5" t="n"/>
-      <c r="I13" s="12">
+      <c r="I13" s="16">
         <f>IF(H13="","",G13/H13)</f>
         <v/>
       </c>
@@ -1697,7 +2037,7 @@
       <c r="F14" s="7" t="n"/>
       <c r="G14" s="5" t="n"/>
       <c r="H14" s="5" t="n"/>
-      <c r="I14" s="12">
+      <c r="I14" s="16">
         <f>IF(H14="","",G14/H14)</f>
         <v/>
       </c>
@@ -1713,7 +2053,7 @@
       <c r="F15" s="7" t="n"/>
       <c r="G15" s="5" t="n"/>
       <c r="H15" s="5" t="n"/>
-      <c r="I15" s="12">
+      <c r="I15" s="16">
         <f>IF(H15="","",G15/H15)</f>
         <v/>
       </c>
@@ -1729,7 +2069,7 @@
       <c r="F16" s="7" t="n"/>
       <c r="G16" s="5" t="n"/>
       <c r="H16" s="5" t="n"/>
-      <c r="I16" s="12">
+      <c r="I16" s="16">
         <f>IF(H16="","",G16/H16)</f>
         <v/>
       </c>
@@ -1745,7 +2085,7 @@
       <c r="F17" s="7" t="n"/>
       <c r="G17" s="5" t="n"/>
       <c r="H17" s="5" t="n"/>
-      <c r="I17" s="12">
+      <c r="I17" s="16">
         <f>IF(H17="","",G17/H17)</f>
         <v/>
       </c>
@@ -1761,7 +2101,7 @@
       <c r="F18" s="7" t="n"/>
       <c r="G18" s="5" t="n"/>
       <c r="H18" s="5" t="n"/>
-      <c r="I18" s="12">
+      <c r="I18" s="16">
         <f>IF(H18="","",G18/H18)</f>
         <v/>
       </c>
@@ -1777,7 +2117,7 @@
       <c r="F19" s="7" t="n"/>
       <c r="G19" s="5" t="n"/>
       <c r="H19" s="5" t="n"/>
-      <c r="I19" s="12">
+      <c r="I19" s="16">
         <f>IF(H19="","",G19/H19)</f>
         <v/>
       </c>
@@ -1793,7 +2133,7 @@
       <c r="F20" s="7" t="n"/>
       <c r="G20" s="5" t="n"/>
       <c r="H20" s="5" t="n"/>
-      <c r="I20" s="12">
+      <c r="I20" s="16">
         <f>IF(H20="","",G20/H20)</f>
         <v/>
       </c>
@@ -1809,7 +2149,7 @@
       <c r="F21" s="7" t="n"/>
       <c r="G21" s="5" t="n"/>
       <c r="H21" s="5" t="n"/>
-      <c r="I21" s="12">
+      <c r="I21" s="16">
         <f>IF(H21="","",G21/H21)</f>
         <v/>
       </c>
@@ -1825,7 +2165,7 @@
       <c r="F22" s="7" t="n"/>
       <c r="G22" s="5" t="n"/>
       <c r="H22" s="5" t="n"/>
-      <c r="I22" s="12">
+      <c r="I22" s="16">
         <f>IF(H22="","",G22/H22)</f>
         <v/>
       </c>
@@ -1841,7 +2181,7 @@
       <c r="F23" s="7" t="n"/>
       <c r="G23" s="5" t="n"/>
       <c r="H23" s="5" t="n"/>
-      <c r="I23" s="12">
+      <c r="I23" s="16">
         <f>IF(H23="","",G23/H23)</f>
         <v/>
       </c>
@@ -1857,7 +2197,7 @@
       <c r="F24" s="7" t="n"/>
       <c r="G24" s="5" t="n"/>
       <c r="H24" s="5" t="n"/>
-      <c r="I24" s="12">
+      <c r="I24" s="16">
         <f>IF(H24="","",G24/H24)</f>
         <v/>
       </c>
@@ -1873,7 +2213,7 @@
       <c r="F25" s="7" t="n"/>
       <c r="G25" s="5" t="n"/>
       <c r="H25" s="5" t="n"/>
-      <c r="I25" s="12">
+      <c r="I25" s="16">
         <f>IF(H25="","",G25/H25)</f>
         <v/>
       </c>
@@ -1889,7 +2229,7 @@
       <c r="F26" s="7" t="n"/>
       <c r="G26" s="5" t="n"/>
       <c r="H26" s="5" t="n"/>
-      <c r="I26" s="12">
+      <c r="I26" s="16">
         <f>IF(H26="","",G26/H26)</f>
         <v/>
       </c>
@@ -1905,7 +2245,7 @@
       <c r="F27" s="7" t="n"/>
       <c r="G27" s="5" t="n"/>
       <c r="H27" s="5" t="n"/>
-      <c r="I27" s="12">
+      <c r="I27" s="16">
         <f>IF(H27="","",G27/H27)</f>
         <v/>
       </c>
@@ -1921,7 +2261,7 @@
       <c r="F28" s="7" t="n"/>
       <c r="G28" s="5" t="n"/>
       <c r="H28" s="5" t="n"/>
-      <c r="I28" s="12">
+      <c r="I28" s="16">
         <f>IF(H28="","",G28/H28)</f>
         <v/>
       </c>
@@ -1937,7 +2277,7 @@
       <c r="F29" s="7" t="n"/>
       <c r="G29" s="5" t="n"/>
       <c r="H29" s="5" t="n"/>
-      <c r="I29" s="12">
+      <c r="I29" s="16">
         <f>IF(H29="","",G29/H29)</f>
         <v/>
       </c>
@@ -1953,7 +2293,7 @@
       <c r="F30" s="7" t="n"/>
       <c r="G30" s="5" t="n"/>
       <c r="H30" s="5" t="n"/>
-      <c r="I30" s="12">
+      <c r="I30" s="16">
         <f>IF(H30="","",G30/H30)</f>
         <v/>
       </c>
@@ -1969,7 +2309,7 @@
       <c r="F31" s="7" t="n"/>
       <c r="G31" s="5" t="n"/>
       <c r="H31" s="5" t="n"/>
-      <c r="I31" s="12">
+      <c r="I31" s="16">
         <f>IF(H31="","",G31/H31)</f>
         <v/>
       </c>
@@ -1985,7 +2325,7 @@
       <c r="F32" s="7" t="n"/>
       <c r="G32" s="5" t="n"/>
       <c r="H32" s="5" t="n"/>
-      <c r="I32" s="12">
+      <c r="I32" s="16">
         <f>IF(H32="","",G32/H32)</f>
         <v/>
       </c>
@@ -2001,7 +2341,7 @@
       <c r="F33" s="7" t="n"/>
       <c r="G33" s="5" t="n"/>
       <c r="H33" s="5" t="n"/>
-      <c r="I33" s="12">
+      <c r="I33" s="16">
         <f>IF(H33="","",G33/H33)</f>
         <v/>
       </c>
@@ -2017,7 +2357,7 @@
       <c r="F34" s="7" t="n"/>
       <c r="G34" s="5" t="n"/>
       <c r="H34" s="5" t="n"/>
-      <c r="I34" s="12">
+      <c r="I34" s="16">
         <f>IF(H34="","",G34/H34)</f>
         <v/>
       </c>
@@ -2033,7 +2373,7 @@
       <c r="F35" s="7" t="n"/>
       <c r="G35" s="5" t="n"/>
       <c r="H35" s="5" t="n"/>
-      <c r="I35" s="12">
+      <c r="I35" s="16">
         <f>IF(H35="","",G35/H35)</f>
         <v/>
       </c>
@@ -2049,7 +2389,7 @@
       <c r="F36" s="7" t="n"/>
       <c r="G36" s="5" t="n"/>
       <c r="H36" s="5" t="n"/>
-      <c r="I36" s="12">
+      <c r="I36" s="16">
         <f>IF(H36="","",G36/H36)</f>
         <v/>
       </c>
@@ -2065,7 +2405,7 @@
       <c r="F37" s="7" t="n"/>
       <c r="G37" s="5" t="n"/>
       <c r="H37" s="5" t="n"/>
-      <c r="I37" s="12">
+      <c r="I37" s="16">
         <f>IF(H37="","",G37/H37)</f>
         <v/>
       </c>
@@ -2081,7 +2421,7 @@
       <c r="F38" s="7" t="n"/>
       <c r="G38" s="5" t="n"/>
       <c r="H38" s="5" t="n"/>
-      <c r="I38" s="12">
+      <c r="I38" s="16">
         <f>IF(H38="","",G38/H38)</f>
         <v/>
       </c>
@@ -2097,7 +2437,7 @@
       <c r="F39" s="7" t="n"/>
       <c r="G39" s="5" t="n"/>
       <c r="H39" s="5" t="n"/>
-      <c r="I39" s="12">
+      <c r="I39" s="16">
         <f>IF(H39="","",G39/H39)</f>
         <v/>
       </c>
@@ -2113,7 +2453,7 @@
       <c r="F40" s="7" t="n"/>
       <c r="G40" s="5" t="n"/>
       <c r="H40" s="5" t="n"/>
-      <c r="I40" s="12">
+      <c r="I40" s="16">
         <f>IF(H40="","",G40/H40)</f>
         <v/>
       </c>
@@ -2129,7 +2469,7 @@
       <c r="F41" s="7" t="n"/>
       <c r="G41" s="5" t="n"/>
       <c r="H41" s="5" t="n"/>
-      <c r="I41" s="12">
+      <c r="I41" s="16">
         <f>IF(H41="","",G41/H41)</f>
         <v/>
       </c>
@@ -2145,7 +2485,7 @@
       <c r="F42" s="7" t="n"/>
       <c r="G42" s="5" t="n"/>
       <c r="H42" s="5" t="n"/>
-      <c r="I42" s="12">
+      <c r="I42" s="16">
         <f>IF(H42="","",G42/H42)</f>
         <v/>
       </c>
@@ -2161,7 +2501,7 @@
       <c r="F43" s="7" t="n"/>
       <c r="G43" s="5" t="n"/>
       <c r="H43" s="5" t="n"/>
-      <c r="I43" s="12">
+      <c r="I43" s="16">
         <f>IF(H43="","",G43/H43)</f>
         <v/>
       </c>
@@ -2177,7 +2517,7 @@
       <c r="F44" s="7" t="n"/>
       <c r="G44" s="5" t="n"/>
       <c r="H44" s="5" t="n"/>
-      <c r="I44" s="12">
+      <c r="I44" s="16">
         <f>IF(H44="","",G44/H44)</f>
         <v/>
       </c>
@@ -2193,7 +2533,7 @@
       <c r="F45" s="7" t="n"/>
       <c r="G45" s="5" t="n"/>
       <c r="H45" s="5" t="n"/>
-      <c r="I45" s="12">
+      <c r="I45" s="16">
         <f>IF(H45="","",G45/H45)</f>
         <v/>
       </c>
@@ -2209,7 +2549,7 @@
       <c r="F46" s="7" t="n"/>
       <c r="G46" s="5" t="n"/>
       <c r="H46" s="5" t="n"/>
-      <c r="I46" s="12">
+      <c r="I46" s="16">
         <f>IF(H46="","",G46/H46)</f>
         <v/>
       </c>
@@ -2225,7 +2565,7 @@
       <c r="F47" s="7" t="n"/>
       <c r="G47" s="5" t="n"/>
       <c r="H47" s="5" t="n"/>
-      <c r="I47" s="12">
+      <c r="I47" s="16">
         <f>IF(H47="","",G47/H47)</f>
         <v/>
       </c>
@@ -2241,7 +2581,7 @@
       <c r="F48" s="7" t="n"/>
       <c r="G48" s="5" t="n"/>
       <c r="H48" s="5" t="n"/>
-      <c r="I48" s="12">
+      <c r="I48" s="16">
         <f>IF(H48="","",G48/H48)</f>
         <v/>
       </c>
@@ -2257,7 +2597,7 @@
       <c r="F49" s="7" t="n"/>
       <c r="G49" s="5" t="n"/>
       <c r="H49" s="5" t="n"/>
-      <c r="I49" s="12">
+      <c r="I49" s="16">
         <f>IF(H49="","",G49/H49)</f>
         <v/>
       </c>
@@ -2273,7 +2613,7 @@
       <c r="F50" s="7" t="n"/>
       <c r="G50" s="5" t="n"/>
       <c r="H50" s="5" t="n"/>
-      <c r="I50" s="12">
+      <c r="I50" s="16">
         <f>IF(H50="","",G50/H50)</f>
         <v/>
       </c>
@@ -2289,7 +2629,7 @@
       <c r="F51" s="7" t="n"/>
       <c r="G51" s="5" t="n"/>
       <c r="H51" s="5" t="n"/>
-      <c r="I51" s="12">
+      <c r="I51" s="16">
         <f>IF(H51="","",G51/H51)</f>
         <v/>
       </c>
@@ -2305,7 +2645,7 @@
       <c r="F52" s="7" t="n"/>
       <c r="G52" s="5" t="n"/>
       <c r="H52" s="5" t="n"/>
-      <c r="I52" s="12">
+      <c r="I52" s="16">
         <f>IF(H52="","",G52/H52)</f>
         <v/>
       </c>
@@ -2321,7 +2661,7 @@
       <c r="F53" s="7" t="n"/>
       <c r="G53" s="5" t="n"/>
       <c r="H53" s="5" t="n"/>
-      <c r="I53" s="12">
+      <c r="I53" s="16">
         <f>IF(H53="","",G53/H53)</f>
         <v/>
       </c>
@@ -2337,7 +2677,7 @@
       <c r="F54" s="7" t="n"/>
       <c r="G54" s="5" t="n"/>
       <c r="H54" s="5" t="n"/>
-      <c r="I54" s="12">
+      <c r="I54" s="16">
         <f>IF(H54="","",G54/H54)</f>
         <v/>
       </c>
@@ -2353,7 +2693,7 @@
       <c r="F55" s="7" t="n"/>
       <c r="G55" s="5" t="n"/>
       <c r="H55" s="5" t="n"/>
-      <c r="I55" s="12">
+      <c r="I55" s="16">
         <f>IF(H55="","",G55/H55)</f>
         <v/>
       </c>
@@ -2369,7 +2709,7 @@
       <c r="F56" s="7" t="n"/>
       <c r="G56" s="5" t="n"/>
       <c r="H56" s="5" t="n"/>
-      <c r="I56" s="12">
+      <c r="I56" s="16">
         <f>IF(H56="","",G56/H56)</f>
         <v/>
       </c>

</xml_diff>